<commit_message>
Keep RibORF IDs and types apart from Chang's; leave out 1-4 residue ORFs
Review of #86 found that naming RibORF ORFs exactly as Chang et al. name
theirs made 78 of Chang's IDs ambiguous or renamed in the merged mouse
catalogue, and that 11,902 imported "proteins" had 1-4 residues (4,386 a
bare M). RibORF IDs now start riborf_, proteins shorter than Chang's
shortest (5 residues) are left out and counted, and ouORF, odORF and
noncoding take Chang's names uoORF, doORF and lncORF. TEC transcripts
with no sequence get their own reason. The fixtures cover the ncRNA
FASTA, every unresolved reason, the length floor and shared-locus IDs.

Merged mouse: 48,805 ORFs; every ID finds its ORF; load 0.9 GB, not 1.1.

Claude-Session: https://claude.ai/code/session_016N35AjLGwyYtEcjeN5k6mT
</commit_message>
<xml_diff>
--- a/tests/data/riborf/SD3.xlsx
+++ b/tests/data/riborf/SD3.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:L19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -784,6 +784,512 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>3</v>
+      </c>
+      <c r="B9" t="n">
+        <v>108112588</v>
+      </c>
+      <c r="C9" t="n">
+        <v>108112594</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>ENSMUST00000000001.4:3:-|62|3262:740:746|iORF|ATG</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>108112588</v>
+      </c>
+      <c r="H9" t="n">
+        <v>108112594</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" t="n">
+        <v>1</v>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>6,</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>0,</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" t="n">
+        <v>41543616</v>
+      </c>
+      <c r="C10" t="n">
+        <v>41543631</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>ENSMUST00000169595.1:6:+|2|48:20:35|noncoding|TTG</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>41543616</v>
+      </c>
+      <c r="H10" t="n">
+        <v>41543631</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" t="n">
+        <v>1</v>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>15,</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>0,</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>13</v>
+      </c>
+      <c r="B11" t="n">
+        <v>4382678</v>
+      </c>
+      <c r="C11" t="n">
+        <v>4382696</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>ENSMUST00000220926.1:13:-|1|166:1:19|noncoding|CTG</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>4382678</v>
+      </c>
+      <c r="H11" t="n">
+        <v>4382696</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" t="n">
+        <v>1</v>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>18,</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>0,</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>18</v>
+      </c>
+      <c r="B12" t="n">
+        <v>57316436</v>
+      </c>
+      <c r="C12" t="n">
+        <v>57316517</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>ENSMUST00000235655.1:18:+|5|279:41:122|noncoding|ACG</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>57316436</v>
+      </c>
+      <c r="H12" t="n">
+        <v>57316517</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" t="n">
+        <v>1</v>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>81,</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>0,</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>2</v>
+      </c>
+      <c r="B13" t="n">
+        <v>11013821</v>
+      </c>
+      <c r="C13" t="n">
+        <v>11013866</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>ENSMUST00000192542.1:2:-|4|111:53:98|noncoding|CTG</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>11013821</v>
+      </c>
+      <c r="H13" t="n">
+        <v>11013866</v>
+      </c>
+      <c r="I13" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" t="n">
+        <v>1</v>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>45,</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>0,</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>14</v>
+      </c>
+      <c r="B14" t="n">
+        <v>8214779</v>
+      </c>
+      <c r="C14" t="n">
+        <v>8214902</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>ENSMUST00000170111.1:14:+|29|3052:279:402|uORF|ATG</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="G14" t="n">
+        <v>8214779</v>
+      </c>
+      <c r="H14" t="n">
+        <v>8214902</v>
+      </c>
+      <c r="I14" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" t="n">
+        <v>1</v>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>123,</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>0,</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="n">
+        <v>8220200</v>
+      </c>
+      <c r="C15" t="n">
+        <v>8222187</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>ENSMUST00000170111.1:14:+|160|3052:1658:1679|iORF|ATG</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="G15" t="n">
+        <v>8220200</v>
+      </c>
+      <c r="H15" t="n">
+        <v>8222187</v>
+      </c>
+      <c r="I15" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" t="n">
+        <v>2</v>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>20,1,</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>0,1986,</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>4</v>
+      </c>
+      <c r="B16" t="n">
+        <v>120447148</v>
+      </c>
+      <c r="C16" t="n">
+        <v>120462104</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>ENSMUST00000000087.12:4:+|14|3353:267:459|ouORF|ATG</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="G16" t="n">
+        <v>120447148</v>
+      </c>
+      <c r="H16" t="n">
+        <v>120462104</v>
+      </c>
+      <c r="I16" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" t="n">
+        <v>4</v>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>13,63,24,92,</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>0,6095,6603,14864,</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" t="n">
+        <v>23745051</v>
+      </c>
+      <c r="C17" t="n">
+        <v>23745087</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>ENSMUST00000091752.4:13:-|29|630:516:552|odORF|ATG</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G17" t="n">
+        <v>23745051</v>
+      </c>
+      <c r="H17" t="n">
+        <v>23745087</v>
+      </c>
+      <c r="I17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>36,</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>0,</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>15</v>
+      </c>
+      <c r="B18" t="n">
+        <v>97361217</v>
+      </c>
+      <c r="C18" t="n">
+        <v>97384062</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>ENSMUST00000226495.1:15:+|1|441:2:155|uORF|ATG</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="G18" t="n">
+        <v>97361217</v>
+      </c>
+      <c r="H18" t="n">
+        <v>97384062</v>
+      </c>
+      <c r="I18" t="n">
+        <v>0</v>
+      </c>
+      <c r="J18" t="n">
+        <v>2</v>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>118,35,</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>0,22810,</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" t="n">
+        <v>97361217</v>
+      </c>
+      <c r="C19" t="n">
+        <v>97384062</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>ENSMUST00000228521.1:15:+|2|1790:17:173|uORF|ATG</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="G19" t="n">
+        <v>97361217</v>
+      </c>
+      <c r="H19" t="n">
+        <v>97384062</v>
+      </c>
+      <c r="I19" t="n">
+        <v>0</v>
+      </c>
+      <c r="J19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>118,38,</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>0,22807,</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>